<commit_message>
Atualização 2 do dia 16/06/2026, adicionada a funcionalidade de remover, e a planilha foi atualizada para fornecer mais informações, assim como a IA também. Funcionalidades ainda não testadas completamente.
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -413,78 +413,60 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Dia</t>
+          <t>Data do registro</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Mês</t>
+          <t>Descrição</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Ano</t>
+          <t>Valor</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Descrição</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Data</t>
+          <t>Dia de Pagamento</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Compra de peça de computador</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>300</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Assinatura</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>16-06-2026</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Conta de Luz</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>200</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>20-06-2026</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
atualização 17/06 - Acabou! o MVP ta pronto
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,11 +442,31 @@
           <t>Dia de Pagamento</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Reserva de Emergência</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Aporte Mensal</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Viver de Renda</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>16-06-2026</t>
+          <t>17-06-2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -454,19 +474,68 @@
           <t>Conta de Luz</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>200</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>R$ 200.00</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Conta</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>21-06-2026</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>R$ 3000</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>R$ 18000</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>R$ 600</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>R$ 360000</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>17-06-2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Lanche iFood</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>R$ 50.00</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>20-06-2026</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Muita coisa, muitos problemas que felizmente foram corrigidos e a salvação chamada Copilot, a interface está feita e alguns % funcional
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,39 +491,31 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>R$ 1000</t>
+          <t>R$ 2000</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> R$ 6000</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>R$ 200</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>R$ 120000</t>
-        </is>
-      </c>
+          <t xml:space="preserve"> R$ 18000</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>03-06-2026</t>
+          <t>04-06-2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Conta de Luz</t>
+          <t>Conta de Água</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>R$ 185</t>
+          <t>R$ 78</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -544,17 +536,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>04-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Conta de Água</t>
+          <t>Internet</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>R$ 78</t>
+          <t>R$ 120</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -564,7 +556,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>12-06-2026</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -575,17 +567,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>06-06-2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Internet</t>
+          <t>Mercado</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>R$ 120</t>
+          <t>R$ 340</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -595,7 +587,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>15-06-2026</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -606,17 +598,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>06-06-2026</t>
+          <t>08-06-2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mercado</t>
+          <t>Lanche</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>R$ 340</t>
+          <t>R$ 25</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -626,7 +618,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15-06-2026</t>
+          <t>08-06-2026</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -637,17 +629,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>08-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Lanche</t>
+          <t>Gasolina</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>R$ 25</t>
+          <t>R$ 180</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -657,7 +649,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>08-06-2026</t>
+          <t>11-06-2026</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -668,27 +660,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>12-06-2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Gasolina</t>
+          <t>Freelance</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>R$ 180</t>
+          <t>R$ 300</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>11-06-2026</t>
+          <t>12-06-2026</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -699,27 +691,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>15-06-2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Freelance</t>
+          <t>Academia</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>R$ 300</t>
+          <t>R$ 89</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Entrada</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>15-06-2026</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -730,17 +722,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>15-06-2026</t>
+          <t>17-06-2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Academia</t>
+          <t>Streaming</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>R$ 89</t>
+          <t>R$ 35</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -750,7 +742,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>15-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -761,17 +753,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>17-06-2026</t>
+          <t>20-06-2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Streaming</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>R$ 35</t>
+          <t>R$ 100</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -781,7 +773,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>20-06-2026</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -792,27 +784,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>20-06-2026</t>
+          <t>22-06-2026</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Presente</t>
+          <t>Venda de Produto</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>R$ 100</t>
+          <t>R$ 450</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>20-06-2026</t>
+          <t>22-06-2026</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -823,181 +815,30 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>22-06-2026</t>
+          <t>09-08-2026</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Venda de Produto</t>
+          <t>Lanche</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>R$ 450</t>
+          <t>R$ 50.00</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Entrada</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>22-06-2026</t>
-        </is>
-      </c>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>25-06-2026</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Telefone</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>R$ 55</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Saída</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>25-06-2026</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>28-06-2026</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Reserva de Emergência</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>R$ 200</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Saída</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>30-06-2026</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>18-06-2026</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Lanche</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>R$ 50</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Saída</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Muitas e poucas mudanças
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -839,6 +839,276 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>09-08-2026</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Lanche McDonalds</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>R$ 50.00</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>09-08-2026</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>McDonald's</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>R$ 50.00</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>09-08-2026</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Lanche McDonalds</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>R$ 50.00</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>09-08-2026</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Lanche McDonalds</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>R$ 50.00</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>09-08-2026</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>McDonald's Lanche</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>R$ 50.00</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>09-08-2026</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Cinema</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>R$ 50.00</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>09-08-2026</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>cinema</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>R$ 50.00</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>09-08-2026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>R$ 100.00</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>09-08-2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Roupas</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>R$ 200</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>09-08-2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Conta a pagar</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>10-08-2026</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
sei nao, to com sono
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,17 +466,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>02-06-2026</t>
+          <t>01/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Vale Transporte</t>
+          <t>Salário</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>R$ 220</t>
+          <t>R$ 5500.00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -484,13 +484,11 @@
           <t>Entrada</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>05-06-2026</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1500</v>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>5500</t>
+        </is>
       </c>
       <c r="G2" t="n">
         <v>18000</v>
@@ -505,17 +503,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>04-06-2026</t>
+          <t>01/08/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Conta de Água</t>
+          <t>Aluguel</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>R$ 78</t>
+          <t>R$ 1500.00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -525,7 +523,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>05/08/2026</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -536,17 +534,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>09-08-2026</t>
+          <t>02/08/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cinema</t>
+          <t>Supermercado</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>R$ 300</t>
+          <t>R$450.00</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -563,17 +561,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>08-08-2026</t>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cinema</t>
+          <t>Conta de Luz</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>R$ 300</t>
+          <t>R$180.00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -581,7 +579,11 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
@@ -590,17 +592,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>09-08-2026</t>
+          <t>04/08/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Roupas</t>
+          <t>Internet</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>R$ 500</t>
+          <t>R$120.00</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -608,12 +610,754 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05/08/2027</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Condomínio</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>R$120.00</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06/08/2026</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Restaurante</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>R$600.00</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>08/08/2026</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>R$150.00</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>10/08/2028</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Freelance de Design</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>R$45.00</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Farmácia</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>R$800.00</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>15/08/2026</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mensalidade Academia</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>R$85.00</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>20/08/2026</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>16/08/2029</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Cinema e Pipoca</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>R$110.00</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Plano de Saúde</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>R$60.00</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>20/08/2026</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Posto de Combustível</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>R$350.00</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>22/08/2030</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Venda de Bicicleta</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>R$200.00</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Assinatura Streaming</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>R$400.00</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Supermercado</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>R$45.00</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>26/08/2026</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Conta de Água</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>R$320.00</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Pet Shop</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>R$95.00</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>30/08/2026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Manutenção do Carro</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>R$130.00</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>R$500.00</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Presente de Aniversário</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>R$5500.00</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>IPTU</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>R$250.00</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saída </t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>15/09/2026</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Café na Padaria</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>R$150.00</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Seguro Auto</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>R$25.00</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>12/09/2026</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Curso Online</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>R$150.00</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>15/09/2026</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>11/09/2034</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Compra de Roupas</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>R$25.00</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Consulta Médica</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>R$220.00</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Reembolso do Plano</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>R$90.00</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>18/09/2035</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Dentista</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>R$350.00</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>20/09/2026</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>IPVA</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>R$250.00</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização do dia 16/08/2026, adicionei a conversaç
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,42 +484,38 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="G2" t="n">
-        <v>120000</v>
+        <v>30000</v>
       </c>
       <c r="H2" t="n">
-        <v>2400000</v>
+        <v>600000</v>
       </c>
       <c r="I2" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>01/08/2026</t>
+          <t>02/08/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Aluguel</t>
+          <t>Supermercado</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1500</v>
+        <v>450</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>05/08/2026</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
@@ -528,23 +524,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>02/08/2026</t>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Supermercado</t>
+          <t>Conta de Luz</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>450</v>
+        <v>180</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
@@ -553,16 +553,16 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
+          <t>04/08/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Conta de Luz</t>
+          <t>Internet</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>180</v>
+        <v>120</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -582,12 +582,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04/08/2026</t>
+          <t>05/08/2027</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Internet</t>
+          <t>Condomínio</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -611,27 +611,23 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05/08/2027</t>
+          <t>06/08/2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Condomínio</t>
+          <t>Restaurante</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>120</v>
+        <v>600</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>10/08/2026</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
@@ -640,16 +636,16 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06/08/2026</t>
+          <t>08/08/2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Restaurante</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>600</v>
+        <v>150</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -665,20 +661,20 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>08/08/2026</t>
+          <t>10/08/2028</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>Freelance de Design</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>150</v>
+        <v>45</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -690,20 +686,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>10/08/2028</t>
+          <t>12/08/2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Freelance de Design</t>
+          <t>Farmácia</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>45</v>
+        <v>800</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Entrada</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -715,23 +711,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/08/2026</t>
+          <t>15/08/2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Farmácia</t>
+          <t>Mensalidade Academia</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>800</v>
+        <v>85</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>20/08/2026</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
@@ -740,27 +740,23 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>15/08/2026</t>
+          <t>16/08/2029</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mensalidade Academia</t>
+          <t>Cinema e Pipoca</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>85</v>
+        <v>110</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>20/08/2026</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -769,23 +765,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>16/08/2029</t>
+          <t>18/08/2026</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cinema e Pipoca</t>
+          <t>Plano de Saúde</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
@@ -794,27 +794,23 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>18/08/2026</t>
+          <t>20/08/2026</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Plano de Saúde</t>
+          <t>Posto de Combustível</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>60</v>
+        <v>350</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>25/08/2026</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
@@ -823,20 +819,20 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>20/08/2026</t>
+          <t>22/08/2030</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Posto de Combustível</t>
+          <t>Venda de Bicicleta</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>350</v>
+        <v>200</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -848,23 +844,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>22/08/2030</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Venda de Bicicleta</t>
+          <t>Assinatura Streaming</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Entrada</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -873,27 +873,23 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>24/08/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Assinatura Streaming</t>
+          <t>Supermercado</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>400</v>
+        <v>45</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>28/08/2026</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
@@ -902,23 +898,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>25/08/2026</t>
+          <t>26/08/2026</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Supermercado</t>
+          <t>Conta de Água</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>45</v>
+        <v>320</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -927,27 +927,23 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>28/08/2026</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Conta de Água</t>
+          <t>Pet Shop</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>320</v>
+        <v>95</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>05/09/2026</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
@@ -956,16 +952,16 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>28/08/2026</t>
+          <t>30/08/2026</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Pet Shop</t>
+          <t>Manutenção do Carro</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>95</v>
+        <v>130</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -981,20 +977,20 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>30/08/2026</t>
+          <t>01/09/2026</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Manutenção do Carro</t>
+          <t>Salário</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>130</v>
+        <v>500</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -1006,20 +1002,20 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>01/09/2026</t>
+          <t>02/09/2026</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Salário</t>
+          <t>Presente de Aniversário</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>500</v>
+        <v>5500</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Entrada</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
@@ -1031,23 +1027,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>03/09/2026</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Presente de Aniversário</t>
+          <t>IPTU</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>5500</v>
+        <v>250</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Saída</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
+          <t xml:space="preserve">Saída </t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>15/09/2026</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -1056,27 +1056,23 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>03/09/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>IPTU</t>
+          <t>Café na Padaria</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Saída </t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>15/09/2026</t>
-        </is>
-      </c>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
@@ -1085,23 +1081,27 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>07/09/2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Café na Padaria</t>
+          <t>Seguro Auto</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>150</v>
+        <v>25</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>12/09/2026</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
@@ -1110,16 +1110,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Seguro Auto</t>
+          <t>Curso Online</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>12/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -1139,27 +1139,23 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2034</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Curso Online</t>
+          <t>Compra de Roupas</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>150</v>
+        <v>25</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>15/09/2026</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
@@ -1168,16 +1164,16 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>11/09/2034</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Compra de Roupas</t>
+          <t>Consulta Médica</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>25</v>
+        <v>220</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1193,20 +1189,20 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Consulta Médica</t>
+          <t>Reembolso do Plano</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>220</v>
+        <v>90</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -1218,20 +1214,20 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>18/09/2035</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Reembolso do Plano</t>
+          <t>Dentista</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>90</v>
+        <v>350</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Entrada</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -1243,23 +1239,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>18/09/2035</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dentista</t>
+          <t>IPVA</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>350</v>
+        <v>250</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
@@ -1268,16 +1268,16 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>16/08/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>IPVA</t>
+          <t>Aluguel</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>250</v>
+        <v>1100</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>20/08/2026</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -1294,131 +1294,6 @@
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>09-08-2026</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Gasto pessoal</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>200</v>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Saída</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>09-08-2026</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Lanche</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>50</v>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Saída</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>10-08-2026</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Lanche</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>20</v>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Saída</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>12/08/2026</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Lanche</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>50</v>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Saída</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>12/08/2026</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Roupas</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>100</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Saída</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização 17/08, coisas novas adicionadas e nenhum bug(acho)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,7 +484,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="G2" t="n">
         <v>30000</v>
@@ -977,20 +977,20 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>01/09/2026</t>
+          <t>02/09/2026</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Salário</t>
+          <t>Presente de Aniversário</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>500</v>
+        <v>5500</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Entrada</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -1002,23 +1002,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>03/09/2026</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Presente de Aniversário</t>
+          <t>IPTU</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>5500</v>
+        <v>250</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Saída</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
+          <t xml:space="preserve">Saída </t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>15/09/2026</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
@@ -1027,27 +1031,23 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>03/09/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>IPTU</t>
+          <t>Café na Padaria</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Saída </t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>15/09/2026</t>
-        </is>
-      </c>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -1056,23 +1056,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>07/09/2026</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Café na Padaria</t>
+          <t>Seguro Auto</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>150</v>
+        <v>25</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>12/09/2026</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
@@ -1081,16 +1085,16 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Seguro Auto</t>
+          <t>Curso Online</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1099,7 +1103,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>12/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -1110,27 +1114,23 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2034</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Curso Online</t>
+          <t>Compra de Roupas</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>150</v>
+        <v>25</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>15/09/2026</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
@@ -1139,16 +1139,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>11/09/2034</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Compra de Roupas</t>
+          <t>Consulta Médica</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>25</v>
+        <v>220</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1164,20 +1164,20 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Consulta Médica</t>
+          <t>Reembolso do Plano</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>220</v>
+        <v>90</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
@@ -1189,20 +1189,20 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>18/09/2035</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Reembolso do Plano</t>
+          <t>Dentista</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>90</v>
+        <v>350</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Entrada</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -1214,23 +1214,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>18/09/2035</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dentista</t>
+          <t>IPVA</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>350</v>
+        <v>250</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
@@ -1239,16 +1243,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>16/08/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>IPVA</t>
+          <t>Aluguel</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>250</v>
+        <v>1100</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1257,7 +1261,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>20/08/2026</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1265,35 +1269,6 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>16/08/2026</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Aluguel</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>1100</v>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Saída</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>20/08/2026</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização na interface do chat
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1319,6 +1319,31 @@
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>22/08/2026</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>50</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Parte da atualização da interface, fiz somente a aba dos botões.
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -484,19 +484,19 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>5000</v>
+        <v>1000</v>
       </c>
       <c r="G2" t="n">
-        <v>30000</v>
+        <v>6000</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>600000.0</t>
+          <t>120000.0</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>200</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização da interface, agora a tela central
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -484,19 +484,19 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="G2" t="n">
-        <v>6000</v>
+        <v>15000</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>120000.0</t>
+          <t>300000.0</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>500</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização da interface quase completa, so falta corrigir uns bug
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -489,15 +489,11 @@
       <c r="G2" t="n">
         <v>15000</v>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>300000.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
+      <c r="H2" t="n">
+        <v>300000</v>
+      </c>
+      <c r="I2" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Atualizado algumas coisas na tela de informações. Comecei a fazer os gráficos na tela de informações
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,16 @@
           <t>Aporte Mensal</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Entradas</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Despesas</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -494,6 +504,12 @@
       </c>
       <c r="I2" t="n">
         <v>200</v>
+      </c>
+      <c r="J2" t="n">
+        <v>335</v>
+      </c>
+      <c r="K2" t="n">
+        <v>14115</v>
       </c>
     </row>
     <row r="3">
@@ -524,6 +540,8 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -553,6 +571,8 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -582,6 +602,8 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -607,6 +629,8 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -632,6 +656,8 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -657,6 +683,8 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -682,6 +710,8 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -711,6 +741,8 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -736,6 +768,8 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -765,6 +799,8 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -790,6 +826,8 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -815,6 +853,8 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -844,6 +884,8 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -869,6 +911,8 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -898,6 +942,8 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -923,6 +969,8 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -948,6 +996,8 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -973,6 +1023,8 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1002,6 +1054,8 @@
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1027,6 +1081,8 @@
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1056,6 +1112,8 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1085,6 +1143,8 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1110,6 +1170,8 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1135,6 +1197,8 @@
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1160,6 +1224,8 @@
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1185,6 +1251,8 @@
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1214,6 +1282,8 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1243,6 +1313,8 @@
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1268,6 +1340,8 @@
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1293,6 +1367,8 @@
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1318,6 +1394,8 @@
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>